<commit_message>
Read-only Modbus TCP server for the CCI / DT Turkey platform: 305 tags at fixed registers, quality registers, header; register map document and Turkey workbooks filled; status in Settings
</commit_message>
<xml_diff>
--- a/docs/turkey/Solar_Tag_List_Rev.1.2.xlsx
+++ b/docs/turkey/Solar_Tag_List_Rev.1.2.xlsx
@@ -1057,16 +1057,18 @@
           <t>Apparent current L1 N</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n"/>
+      <c r="B2" s="5" t="n">
+        <v>670</v>
+      </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Float</t>
+          <t>Float32 (ABCD)</t>
         </is>
       </c>
       <c r="D2" s="3" t="n"/>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>SAU-100 electric meter (LV PV panel)</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -1076,17 +1078,15 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.128:502</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>TBC (meter address on SAU)</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 2 regs</t>
         </is>
       </c>
       <c r="J2" s="8" t="inlineStr">
@@ -1094,14 +1094,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="K2" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K2" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1290</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -1116,10 +1114,12 @@
           <t>Apparent current L2 N</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n"/>
+      <c r="B3" s="5" t="n">
+        <v>672</v>
+      </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Float</t>
+          <t>Float32 (ABCD)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>SAU-100 electric meter (LV PV panel)</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -1139,17 +1139,15 @@
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.128:502</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>TBC (meter address on SAU)</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 2 regs</t>
         </is>
       </c>
       <c r="J3" s="8" t="inlineStr">
@@ -1157,14 +1155,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K3" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1291</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr"/>
@@ -1175,16 +1171,18 @@
           <t>Apparent current L3 N</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n"/>
+      <c r="B4" s="5" t="n">
+        <v>674</v>
+      </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Float</t>
+          <t>Float32 (ABCD)</t>
         </is>
       </c>
       <c r="D4" s="3" t="n"/>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>SAU-100 electric meter (LV PV panel)</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -1194,17 +1192,15 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.128:502</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>TBC (meter address on SAU)</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 2 regs</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
@@ -1212,14 +1208,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K4" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1292</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr"/>
@@ -1230,10 +1224,12 @@
           <t>Psum3</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
+      <c r="B5" s="5" t="n">
+        <v>676</v>
+      </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Float</t>
+          <t>Float32 (ABCD)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1243,7 +1239,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>SAU-100 electric meter (LV PV panel)</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -1253,17 +1249,15 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.128:502</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>TBC (meter address on SAU)</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 2 regs</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
@@ -1271,14 +1265,12 @@
           <t>kW</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K5" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1293</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr">
@@ -1293,10 +1285,12 @@
           <t>Qsum3</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n"/>
+      <c r="B6" s="5" t="n">
+        <v>678</v>
+      </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Float</t>
+          <t>Float32 (ABCD)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -1306,7 +1300,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>SAU-100 electric meter (LV PV panel)</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -1316,17 +1310,15 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.128:502</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>TBC (meter address on SAU)</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 2 regs</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
@@ -1334,14 +1326,12 @@
           <t>kvar</t>
         </is>
       </c>
-      <c r="K6" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K6" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1294</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr"/>
@@ -1352,16 +1342,18 @@
           <t>Real energy L1 L3 delivered</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n"/>
+      <c r="B7" s="5" t="n">
+        <v>680</v>
+      </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Float</t>
+          <t>Float32 (ABCD)</t>
         </is>
       </c>
       <c r="D7" s="3" t="n"/>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>SAU-100 electric meter (LV PV panel)</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -1371,17 +1363,15 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.128:502</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>TBC (meter address on SAU)</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 2 regs</t>
         </is>
       </c>
       <c r="J7" s="8" t="inlineStr">
@@ -1389,14 +1379,12 @@
           <t>kWh</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K7" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1295</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr">
@@ -1411,16 +1399,18 @@
           <t>Voltage L1 N</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n"/>
+      <c r="B8" s="5" t="n">
+        <v>682</v>
+      </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Float</t>
+          <t>Float32 (ABCD)</t>
         </is>
       </c>
       <c r="D8" s="3" t="n"/>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>SAU-100 electric meter (LV PV panel)</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -1430,17 +1420,15 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.128:502</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>TBC (meter address on SAU)</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 2 regs</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
@@ -1448,14 +1436,12 @@
           <t>V</t>
         </is>
       </c>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K8" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1296</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr"/>
@@ -1466,16 +1452,18 @@
           <t>Voltage L2 N</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n"/>
+      <c r="B9" s="5" t="n">
+        <v>684</v>
+      </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Float</t>
+          <t>Float32 (ABCD)</t>
         </is>
       </c>
       <c r="D9" s="3" t="n"/>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>SAU-100 electric meter (LV PV panel)</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -1485,17 +1473,15 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.128:502</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>TBC (meter address on SAU)</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 2 regs</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
@@ -1503,14 +1489,12 @@
           <t>V</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K9" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1297</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr"/>
@@ -1521,16 +1505,18 @@
           <t>Voltage L3 N</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
+      <c r="B10" s="5" t="n">
+        <v>686</v>
+      </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Float</t>
+          <t>Float32 (ABCD)</t>
         </is>
       </c>
       <c r="D10" s="3" t="n"/>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>SAU-100 electric meter (LV PV panel)</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -1540,17 +1526,15 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.128:502</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>TBC (meter address on SAU)</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 2 regs</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
@@ -1558,14 +1542,12 @@
           <t>V</t>
         </is>
       </c>
-      <c r="K10" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K10" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1298</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr"/>
@@ -1576,16 +1558,18 @@
           <t>Panel Temperature</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n"/>
+      <c r="B11" s="5" t="n">
+        <v>688</v>
+      </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Word</t>
+          <t>Float32 (ABCD)</t>
         </is>
       </c>
       <c r="D11" s="3" t="n"/>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>SAU-100 environmental input (weather station) — TBC</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1595,17 +1579,15 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.128:502</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 2 regs</t>
         </is>
       </c>
       <c r="J11" s="8" t="inlineStr">
@@ -1613,14 +1595,12 @@
           <t>°C</t>
         </is>
       </c>
-      <c r="K11" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K11" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1299</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
@@ -1635,16 +1615,18 @@
           <t>Pyranometer</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n"/>
+      <c r="B12" s="5" t="n">
+        <v>690</v>
+      </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Word</t>
+          <t>Float32 (ABCD)</t>
         </is>
       </c>
       <c r="D12" s="3" t="n"/>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>SAU-100 environmental input (weather station) — TBC</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1654,17 +1636,15 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.128:502</t>
-        </is>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 2 regs</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
@@ -1672,14 +1652,12 @@
           <t>W/m²</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K12" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1300</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
@@ -1694,16 +1672,18 @@
           <t>Area_Connection_Error</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n"/>
+      <c r="B13" s="5" t="n">
+        <v>692</v>
+      </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
       <c r="D13" s="3" t="n"/>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>ComAp InteliNeo 5500</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1713,28 +1693,24 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.112:502</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>TBC (InteliNeo Modbus address)</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 1 reg</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr"/>
-      <c r="K13" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K13" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1301</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr">
@@ -1749,16 +1725,18 @@
           <t>Thermal_Magnetic_Switch_On_(LV PANEL)</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n"/>
+      <c r="B14" s="5" t="n">
+        <v>693</v>
+      </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
       <c r="D14" s="3" t="n"/>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>ComAp InteliNeo 5500</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1768,28 +1746,24 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.112:502</t>
-        </is>
-      </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>TBC (InteliNeo Modbus address)</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 1 reg</t>
         </is>
       </c>
       <c r="J14" s="8" t="inlineStr"/>
-      <c r="K14" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K14" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1302</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -1804,16 +1778,18 @@
           <t>Thermal_Magnetic_Switch_Off (LV PANEL)</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n"/>
+      <c r="B15" s="5" t="n">
+        <v>694</v>
+      </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Boolean (uint16 0/1)</t>
         </is>
       </c>
       <c r="D15" s="3" t="n"/>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>ComAp InteliNeo 5500</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1823,28 +1799,24 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.112:502</t>
-        </is>
-      </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>TBC (InteliNeo Modbus address)</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 1 reg</t>
         </is>
       </c>
       <c r="J15" s="8" t="inlineStr"/>
-      <c r="K15" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K15" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L15" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1303</t>
         </is>
       </c>
       <c r="M15" s="8" t="inlineStr">
@@ -1859,16 +1831,18 @@
           <t>Total_Energy</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n"/>
+      <c r="B16" s="5" t="n">
+        <v>695</v>
+      </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Word</t>
+          <t>Float32 (ABCD)</t>
         </is>
       </c>
       <c r="D16" s="3" t="n"/>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>SAU-100 electric meter (LV PV panel)</t>
+          <t>Plant PC data collector (Modbus TCP server, read-only)</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1878,17 +1852,15 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>192.168.0.128:502</t>
-        </is>
-      </c>
-      <c r="H16" s="7" t="inlineStr">
-        <is>
-          <t>TBC (meter address on SAU)</t>
-        </is>
+          <t>&lt;plant-pc-vpn-ip&gt;:502</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Holding (FC03), 2 regs</t>
         </is>
       </c>
       <c r="J16" s="8" t="inlineStr">
@@ -1896,14 +1868,12 @@
           <t>kWh</t>
         </is>
       </c>
-      <c r="K16" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="K16" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>TBC</t>
+          <t>Ready — quality register 1304</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">

</xml_diff>